<commit_message>
docs(enterprise): reconcile snapshot, QA and decision gates
</commit_message>
<xml_diff>
--- a/smartlock-docs/enterprise/規格統控整理/SmartLock_業務邏輯驗收控制表.xlsx
+++ b/smartlock-docs/enterprise/規格統控整理/SmartLock_業務邏輯驗收控制表.xlsx
@@ -942,17 +942,15 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>6/7 有案例</t>
+          <t>7/7 有案例</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>S1：6 案例</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="n">
-        <v>4</v>
-      </c>
+          <t>S1：13 案例</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="6" t="inlineStr"/>
       <c r="P2" s="6" t="inlineStr"/>
       <c r="Q2" s="6" t="inlineStr"/>
@@ -1012,17 +1010,15 @@
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>6/7 有案例</t>
+          <t>7/7 有案例</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>S1：7 案例</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="n">
-        <v>4</v>
-      </c>
+          <t>S1：12 案例</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr"/>
       <c r="O3" s="6" t="inlineStr"/>
       <c r="P3" s="6" t="inlineStr"/>
       <c r="Q3" s="6" t="inlineStr"/>
@@ -1082,17 +1078,15 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>5/6 有案例</t>
+          <t>6/6 有案例</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>S1：4 案例</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="n">
-        <v>1</v>
-      </c>
+          <t>S1：6 案例</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="6" t="inlineStr"/>
       <c r="P4" s="6" t="inlineStr"/>
       <c r="Q4" s="6" t="inlineStr"/>
@@ -1157,12 +1151,10 @@
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>S2：11 案例</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="n">
-        <v>1</v>
-      </c>
+          <t>S2：12 案例</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr"/>
       <c r="O5" s="6" t="inlineStr"/>
       <c r="P5" s="6" t="inlineStr"/>
       <c r="Q5" s="6" t="inlineStr"/>
@@ -1222,17 +1214,15 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>5/7 有案例</t>
+          <t>7/7 有案例</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>S2：6 案例</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>S2：12 案例</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="6" t="inlineStr"/>
       <c r="P6" s="6" t="inlineStr"/>
       <c r="Q6" s="6" t="inlineStr"/>
@@ -1292,17 +1282,15 @@
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>5/6 有案例</t>
+          <t>6/6 有案例</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>S2：9 案例</t>
-        </is>
-      </c>
-      <c r="N7" s="5" t="n">
-        <v>5</v>
-      </c>
+          <t>S2：15 案例</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
@@ -1367,12 +1355,10 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>S2：5 案例</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="n">
-        <v>4</v>
-      </c>
+          <t>S2：7 案例</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="6" t="inlineStr"/>
       <c r="P8" s="6" t="inlineStr"/>
       <c r="Q8" s="6" t="inlineStr"/>
@@ -1437,12 +1423,10 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>S4：8 案例</t>
-        </is>
-      </c>
-      <c r="N9" s="5" t="n">
-        <v>1</v>
-      </c>
+          <t>S4：11 案例</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
@@ -1507,12 +1491,10 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>1 案例</t>
-        </is>
-      </c>
-      <c r="N10" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>4 案例</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="6" t="inlineStr"/>
       <c r="Q10" s="6" t="inlineStr"/>
@@ -1577,12 +1559,10 @@
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>⚠ 無驗收腳本</t>
-        </is>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>1</v>
-      </c>
+          <t>S6：5 案例</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr"/>
       <c r="O11" s="6" t="inlineStr"/>
       <c r="P11" s="6" t="inlineStr"/>
       <c r="Q11" s="6" t="inlineStr"/>
@@ -1647,12 +1627,10 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>S4：2 案例</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="n">
-        <v>3</v>
-      </c>
+          <t>S4：5 案例</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr"/>
       <c r="O12" s="6" t="inlineStr"/>
       <c r="P12" s="6" t="inlineStr"/>
       <c r="Q12" s="6" t="inlineStr"/>
@@ -1712,17 +1690,15 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>2/4 有案例</t>
+          <t>4/4 有案例</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>⚠ 無驗收腳本</t>
-        </is>
-      </c>
-      <c r="N13" s="5" t="n">
-        <v>1</v>
-      </c>
+          <t>S7：6 案例</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr"/>
       <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="6" t="inlineStr"/>
       <c r="Q13" s="6" t="inlineStr"/>
@@ -1787,12 +1763,10 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>1 案例</t>
-        </is>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>3 案例</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr"/>
       <c r="O14" s="6" t="inlineStr"/>
       <c r="P14" s="6" t="inlineStr"/>
       <c r="Q14" s="6" t="inlineStr"/>
@@ -1852,17 +1826,15 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>3/4 有案例</t>
+          <t>4/4 有案例</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>⚠ 無驗收腳本</t>
-        </is>
-      </c>
-      <c r="N15" s="5" t="n">
-        <v>1</v>
-      </c>
+          <t>S8：6 案例</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr"/>
       <c r="O15" s="6" t="inlineStr"/>
       <c r="P15" s="6" t="inlineStr"/>
       <c r="Q15" s="6" t="inlineStr"/>
@@ -1922,17 +1894,15 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>4/9 有案例</t>
+          <t>9/9 有案例</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>S3：1 案例</t>
-        </is>
-      </c>
-      <c r="N16" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>S3：6 案例</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr"/>
       <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="6" t="inlineStr"/>
       <c r="Q16" s="6" t="inlineStr"/>
@@ -1997,12 +1967,10 @@
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>S3：1 案例</t>
-        </is>
-      </c>
-      <c r="N17" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>S3：3 案例</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
@@ -2062,17 +2030,15 @@
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>2/4 有案例</t>
+          <t>4/4 有案例</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>⚠ 無驗收腳本</t>
-        </is>
-      </c>
-      <c r="N18" s="5" t="n">
-        <v>1</v>
-      </c>
+          <t>S9：6 案例</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr"/>
       <c r="O18" s="6" t="inlineStr"/>
       <c r="P18" s="6" t="inlineStr"/>
       <c r="Q18" s="6" t="inlineStr"/>
@@ -2132,17 +2098,15 @@
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>1/4 有案例</t>
+          <t>4/4 有案例</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>S5：1 案例</t>
-        </is>
-      </c>
-      <c r="N19" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>S5：6 案例</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr"/>
       <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="6" t="inlineStr"/>
       <c r="Q19" s="6" t="inlineStr"/>
@@ -2207,12 +2171,10 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>S4：5 案例</t>
-        </is>
-      </c>
-      <c r="N20" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>S4：7 案例</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr"/>
       <c r="O20" s="6" t="inlineStr"/>
       <c r="P20" s="6" t="inlineStr"/>
       <c r="Q20" s="6" t="inlineStr"/>
@@ -2381,7 +2343,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -2428,7 +2390,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>happy、boundary</t>
+          <t>happy、boundary、recovery</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -2475,7 +2437,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -2569,7 +2531,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -2616,7 +2578,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -2663,7 +2625,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -2710,7 +2672,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -2804,7 +2766,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -2851,7 +2813,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2898,7 +2860,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -2992,7 +2954,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>happy、boundary</t>
+          <t>happy、boundary、recovery</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -3133,7 +3095,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -3180,7 +3142,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -3227,7 +3189,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -3274,7 +3236,7 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -3368,7 +3330,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、recovery</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -3556,7 +3518,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -3603,7 +3565,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -3979,7 +3941,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -4167,7 +4129,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -4214,7 +4176,7 @@
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
@@ -4261,7 +4223,7 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -4355,7 +4317,7 @@
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -4496,7 +4458,7 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -4543,7 +4505,7 @@
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
@@ -4590,7 +4552,7 @@
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
@@ -4825,7 +4787,7 @@
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -4872,7 +4834,7 @@
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
@@ -5295,7 +5257,7 @@
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
@@ -5483,7 +5445,7 @@
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
@@ -5671,7 +5633,7 @@
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
@@ -5718,7 +5680,7 @@
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
@@ -5859,7 +5821,7 @@
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
@@ -5953,7 +5915,7 @@
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
@@ -6047,7 +6009,7 @@
       </c>
       <c r="H81" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I81" s="5" t="inlineStr">
@@ -6094,7 +6056,7 @@
       </c>
       <c r="H82" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
@@ -6188,7 +6150,7 @@
       </c>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
@@ -6235,7 +6197,7 @@
       </c>
       <c r="H85" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I85" s="5" t="inlineStr">
@@ -6282,7 +6244,7 @@
       </c>
       <c r="H86" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
@@ -6423,7 +6385,7 @@
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
@@ -6564,7 +6526,7 @@
       </c>
       <c r="H92" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
@@ -6658,7 +6620,7 @@
       </c>
       <c r="H94" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I94" s="5" t="inlineStr">
@@ -6799,7 +6761,7 @@
       </c>
       <c r="H97" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I97" s="5" t="inlineStr">
@@ -6846,7 +6808,7 @@
       </c>
       <c r="H98" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I98" s="5" t="inlineStr">
@@ -6893,7 +6855,7 @@
       </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I99" s="5" t="inlineStr">
@@ -6940,7 +6902,7 @@
       </c>
       <c r="H100" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I100" s="5" t="inlineStr">
@@ -6987,7 +6949,7 @@
       </c>
       <c r="H101" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I101" s="5" t="inlineStr">
@@ -7034,7 +6996,7 @@
       </c>
       <c r="H102" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I102" s="5" t="inlineStr">
@@ -7081,7 +7043,7 @@
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr">
@@ -7128,7 +7090,7 @@
       </c>
       <c r="H104" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I104" s="5" t="inlineStr">
@@ -7175,7 +7137,7 @@
       </c>
       <c r="H105" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I105" s="5" t="inlineStr">
@@ -7222,7 +7184,7 @@
       </c>
       <c r="H106" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I106" s="5" t="inlineStr">
@@ -7269,7 +7231,7 @@
       </c>
       <c r="H107" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I107" s="5" t="inlineStr">
@@ -7316,7 +7278,7 @@
       </c>
       <c r="H108" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I108" s="5" t="inlineStr">
@@ -7363,7 +7325,7 @@
       </c>
       <c r="H109" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I109" s="5" t="inlineStr">
@@ -7410,7 +7372,7 @@
       </c>
       <c r="H110" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I110" s="5" t="inlineStr">
@@ -7457,7 +7419,7 @@
       </c>
       <c r="H111" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I111" s="5" t="inlineStr">
@@ -7504,7 +7466,7 @@
       </c>
       <c r="H112" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I112" s="5" t="inlineStr">
@@ -7551,7 +7513,7 @@
       </c>
       <c r="H113" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I113" s="5" t="inlineStr">
@@ -7598,7 +7560,7 @@
       </c>
       <c r="H114" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I114" s="5" t="inlineStr">
@@ -7645,7 +7607,7 @@
       </c>
       <c r="H115" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I115" s="5" t="inlineStr">
@@ -7692,7 +7654,7 @@
       </c>
       <c r="H116" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I116" s="5" t="inlineStr">
@@ -7739,7 +7701,7 @@
       </c>
       <c r="H117" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I117" s="5" t="inlineStr">
@@ -7786,7 +7748,7 @@
       </c>
       <c r="H118" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I118" s="5" t="inlineStr">
@@ -7833,7 +7795,7 @@
       </c>
       <c r="H119" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I119" s="5" t="inlineStr">
@@ -7927,7 +7889,7 @@
       </c>
       <c r="H121" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I121" s="5" t="inlineStr">
@@ -7974,7 +7936,7 @@
       </c>
       <c r="H122" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I122" s="5" t="inlineStr">
@@ -8021,7 +7983,7 @@
       </c>
       <c r="H123" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I123" s="5" t="inlineStr">
@@ -8068,7 +8030,7 @@
       </c>
       <c r="H124" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I124" s="5" t="inlineStr">
@@ -8115,7 +8077,7 @@
       </c>
       <c r="H125" s="5" t="inlineStr">
         <is>
-          <t>無案例</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I125" s="5" t="inlineStr">
@@ -8256,7 +8218,7 @@
       </c>
       <c r="H128" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="I128" s="5" t="inlineStr">
@@ -8303,7 +8265,7 @@
       </c>
       <c r="H129" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I129" s="5" t="inlineStr">
@@ -8397,7 +8359,7 @@
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>happy、failure</t>
         </is>
       </c>
       <c r="I131" s="5" t="inlineStr">
@@ -8444,7 +8406,7 @@
       </c>
       <c r="H132" s="5" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>failure</t>
         </is>
       </c>
       <c r="I132" s="5" t="inlineStr">

</xml_diff>